<commit_message>
Lab 1 review fixes: consistent R1 metric, stakeholder quadrants, readable sheet views, team parameters
</commit_message>
<xml_diff>
--- a/lab1/out/lab1_passport_model.xlsx
+++ b/lab1/out/lab1_passport_model.xlsx
@@ -39,7 +39,9 @@
     <definedName name="p_support_rate">'Параметри'!$C$21</definedName>
     <definedName name="p_fixed_platform">'Параметри'!$C$22</definedName>
     <definedName name="p_buildings_y3">'Параметри'!$C$23</definedName>
-    <definedName name="p_price_hypothesis">'Параметри'!$C$24</definedName>
+    <definedName name="p_mvp_months">'Параметри'!$C$24</definedName>
+    <definedName name="p_team_size">'Параметри'!$C$25</definedName>
+    <definedName name="p_price_hypothesis">'Параметри'!$C$26</definedName>
     <definedName name="v_unit">'Змінні витрати'!$C$6</definedName>
     <definedName name="f_fixed">'Змінні витрати'!$C$7</definedName>
   </definedNames>
@@ -599,7 +601,7 @@
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>Виявлення аномалії протягом 2 год замість 12 діб і встановлення її причини до рахунку; оцінена цінність 10 800 EUR на будівлю за рік (П)</t>
+          <t>Медіанний час виявлення аномалії не більше 2 год замість 12 діб і встановлення її причини до рахунку; оцінена цінність 10 800 EUR на будівлю за рік (П)</t>
         </is>
       </c>
     </row>
@@ -611,7 +613,7 @@
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>Медіана часу від початку аномалії до її фіксації: база 288 год (П), ціль не більше 2 год для 80% аномалій за 3 міс.</t>
+          <t>Медіана часу від початку аномалії до її фіксації: база 288 год (П), ціль: медіана не більше 2 год за 3 міс. пілоту; додатковий контроль хвоста розподілу: P80 не більше 4 год</t>
         </is>
       </c>
     </row>
@@ -663,7 +665,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:F24"/>
+  <dimension ref="A1:F26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -1369,28 +1371,88 @@
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
+          <t>p_mvp_months</t>
+        </is>
+      </c>
+      <c r="B24" s="2" t="inlineStr">
+        <is>
+          <t>Строк розроблення MVP</t>
+        </is>
+      </c>
+      <c r="C24" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="D24" s="2" t="inlineStr">
+        <is>
+          <t>міс.</t>
+        </is>
+      </c>
+      <c r="E24" s="2" t="inlineStr">
+        <is>
+          <t>Д</t>
+        </is>
+      </c>
+      <c r="F24" s="2" t="inlineStr">
+        <is>
+          <t>умова варіанта ЛР № 4 і № 5</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="2" t="inlineStr">
+        <is>
+          <t>p_team_size</t>
+        </is>
+      </c>
+      <c r="B25" s="2" t="inlineStr">
+        <is>
+          <t>Чисельність команди MVP</t>
+        </is>
+      </c>
+      <c r="C25" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="D25" s="2" t="inlineStr">
+        <is>
+          <t>осіб</t>
+        </is>
+      </c>
+      <c r="E25" s="2" t="inlineStr">
+        <is>
+          <t>Д</t>
+        </is>
+      </c>
+      <c r="F25" s="2" t="inlineStr">
+        <is>
+          <t>умова варіанта ЛР № 4 і № 5: BA/PM, 2 розробники, QA, DevOps</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="2" t="inlineStr">
+        <is>
           <t>p_price_hypothesis</t>
         </is>
       </c>
-      <c r="B24" s="2" t="inlineStr">
+      <c r="B26" s="2" t="inlineStr">
         <is>
           <t>Гіпотеза ціни для перевірки A2</t>
         </is>
       </c>
-      <c r="C24" s="3" t="n">
+      <c r="C26" s="3" t="n">
         <v>130</v>
       </c>
-      <c r="D24" s="2" t="inlineStr">
+      <c r="D26" s="2" t="inlineStr">
         <is>
           <t>EUR/міс</t>
         </is>
       </c>
-      <c r="E24" s="2" t="inlineStr">
+      <c r="E26" s="2" t="inlineStr">
         <is>
           <t>П</t>
         </is>
       </c>
-      <c r="F24" s="2" t="inlineStr">
+      <c r="F26" s="2" t="inlineStr">
         <is>
           <t>не більше 15% оціненої вигоди</t>
         </is>
@@ -1965,17 +2027,18 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:H8"/>
+  <dimension ref="A1:I8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
     <col width="22" customWidth="1" min="2" max="2"/>
     <col width="32" customWidth="1" min="3" max="3"/>
     <col width="9" customWidth="1" min="4" max="4"/>
-    <col width="13" customWidth="1" min="5" max="5"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
     <col width="11" customWidth="1" min="6" max="6"/>
-    <col width="32" customWidth="1" min="7" max="7"/>
-    <col width="30" customWidth="1" min="8" max="8"/>
+    <col width="15" customWidth="1" min="7" max="7"/>
+    <col width="32" customWidth="1" min="8" max="8"/>
+    <col width="30" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2011,10 +2074,15 @@
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
+          <t>Квадрант</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
           <t>Конфлікт, ризик</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>Залучення</t>
         </is>
@@ -2046,12 +2114,16 @@
         <f>D2*E2</f>
         <v/>
       </c>
-      <c r="G2" s="2" t="inlineStr">
+      <c r="G2" s="7">
+        <f>IF(AND(D2&gt;=4,E2&gt;=4),"керувати тісно",IF(D2&gt;=4,"задовольняти",IF(E2&gt;=4,"інформувати","спостерігати")))</f>
+        <v/>
+      </c>
+      <c r="H2" s="2" t="inlineStr">
         <is>
           <t>зростання навантаження через хибні алерти</t>
         </is>
       </c>
-      <c r="H2" s="2" t="inlineStr">
+      <c r="I2" s="2" t="inlineStr">
         <is>
           <t>інтерв'ю, пілот, щотижневий розбір алертів</t>
         </is>
@@ -2083,12 +2155,16 @@
         <f>D3*E3</f>
         <v/>
       </c>
-      <c r="G3" s="2" t="inlineStr">
+      <c r="G3" s="7">
+        <f>IF(AND(D3&gt;=4,E3&gt;=4),"керувати тісно",IF(D3&gt;=4,"задовольняти",IF(E3&gt;=4,"інформувати","спостерігати")))</f>
+        <v/>
+      </c>
+      <c r="H3" s="2" t="inlineStr">
         <is>
           <t>сприймає систему як контроль своєї роботи</t>
         </is>
       </c>
-      <c r="H3" s="2" t="inlineStr">
+      <c r="I3" s="2" t="inlineStr">
         <is>
           <t>навчання 1 год, довідник причин зі слів техніків</t>
         </is>
@@ -2114,18 +2190,22 @@
         <v>5</v>
       </c>
       <c r="E4" s="7" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F4" s="7">
         <f>D4*E4</f>
         <v/>
       </c>
-      <c r="G4" s="2" t="inlineStr">
+      <c r="G4" s="7">
+        <f>IF(AND(D4&gt;=4,E4&gt;=4),"керувати тісно",IF(D4&gt;=4,"задовольняти",IF(E4&gt;=4,"інформувати","спостерігати")))</f>
+        <v/>
+      </c>
+      <c r="H4" s="2" t="inlineStr">
         <is>
           <t>очікує окупність до 12 міс., не готовий фінансувати заміну лічильників</t>
         </is>
       </c>
-      <c r="H4" s="2" t="inlineStr">
+      <c r="I4" s="2" t="inlineStr">
         <is>
           <t>розрахунок економії, лист про намір, звіт пілоту</t>
         </is>
@@ -2157,12 +2237,16 @@
         <f>D5*E5</f>
         <v/>
       </c>
-      <c r="G5" s="2" t="inlineStr">
+      <c r="G5" s="7">
+        <f>IF(AND(D5&gt;=4,E5&gt;=4),"керувати тісно",IF(D5&gt;=4,"задовольняти",IF(E5&gt;=4,"інформувати","спостерігати")))</f>
+        <v/>
+      </c>
+      <c r="H5" s="2" t="inlineStr">
         <is>
           <t>економія зменшує базу винагороди, якщо вона залежить від обсягу витрат</t>
         </is>
       </c>
-      <c r="H5" s="2" t="inlineStr">
+      <c r="I5" s="2" t="inlineStr">
         <is>
           <t>партнерський пілот, спільні KPI</t>
         </is>
@@ -2194,12 +2278,16 @@
         <f>D6*E6</f>
         <v/>
       </c>
-      <c r="G6" s="2" t="inlineStr">
+      <c r="G6" s="7">
+        <f>IF(AND(D6&gt;=4,E6&gt;=4),"керувати тісно",IF(D6&gt;=4,"задовольняти",IF(E6&gt;=4,"інформувати","спостерігати")))</f>
+        <v/>
+      </c>
+      <c r="H6" s="2" t="inlineStr">
         <is>
           <t>небажання розкривати графік роботи, спори щодо розподілу</t>
         </is>
       </c>
-      <c r="H6" s="2" t="inlineStr">
+      <c r="I6" s="2" t="inlineStr">
         <is>
           <t>щомісячний звіт лише по власних лічильниках</t>
         </is>
@@ -2231,12 +2319,16 @@
         <f>D7*E7</f>
         <v/>
       </c>
-      <c r="G7" s="2" t="inlineStr">
+      <c r="G7" s="7">
+        <f>IF(AND(D7&gt;=4,E7&gt;=4),"керувати тісно",IF(D7&gt;=4,"задовольняти",IF(E7&gt;=4,"інформувати","спостерігати")))</f>
+        <v/>
+      </c>
+      <c r="H7" s="2" t="inlineStr">
         <is>
           <t>закриті протоколи, власна хмара як конкурент</t>
         </is>
       </c>
-      <c r="H7" s="2" t="inlineStr">
+      <c r="I7" s="2" t="inlineStr">
         <is>
           <t>запит карти регістрів Modbus, тестовий стенд</t>
         </is>
@@ -2268,12 +2360,16 @@
         <f>D8*E8</f>
         <v/>
       </c>
-      <c r="G8" s="2" t="inlineStr">
+      <c r="G8" s="7">
+        <f>IF(AND(D8&gt;=4,E8&gt;=4),"керувати тісно",IF(D8&gt;=4,"задовольняти",IF(E8&gt;=4,"інформувати","спостерігати")))</f>
+        <v/>
+      </c>
+      <c r="H8" s="2" t="inlineStr">
         <is>
           <t>розбіжність субобліку і комерційного обліку</t>
         </is>
       </c>
-      <c r="H8" s="2" t="inlineStr">
+      <c r="I8" s="2" t="inlineStr">
         <is>
           <t>імпорт рахунків, звірка показів вводу</t>
         </is>
@@ -2496,12 +2592,12 @@
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>Розроблення backend, frontend і ПЗ шлюзу (2 розробники)</t>
+          <t>Розроблення MVP командою з 5 осіб протягом 7 міс.: BA/PM, 2 розробники (backend, frontend, ПЗ шлюзу), QA, DevOps</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>обсяг scope, SP</t>
+          <t>обсяг scope, SP; FTE ролей</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
@@ -2533,7 +2629,7 @@
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>Тестування і тестовий стенд з 6 типами лічильників</t>
+          <t>Тестовий стенд з 6 типами лічильників</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Lab 1 review fixes: A1 threshold value, hourly input data tests, mean and median basis, readable diagrams
</commit_message>
<xml_diff>
--- a/lab1/out/lab1_passport_model.xlsx
+++ b/lab1/out/lab1_passport_model.xlsx
@@ -553,7 +553,7 @@
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Енергоменеджер багатоорендного офісного центру дізнається про аномальне споживання лише з місячного рахунку, у середньому через 12 діб (П); причину перевитрат встановити складно, бо немає інтервальних даних по точках обліку. Втрати від аномалій оцінено в 3,4% річного споживання (П).</t>
+          <t>Енергоменеджер багатоорендного офісного центру виявляє аномальне споживання із запізненням (обходи, погодинні дані вводу або лише місячний рахунок): середнє і медіана 12 діб (П); причину перевитрат встановити складно, бо субоблік знімають вручну раз на місяць, а погодинні дані є лише по вводу, без інтервальних даних по точках обліку. Втрати від аномалій оцінено в 3,4% річного споживання (П).</t>
         </is>
       </c>
     </row>
@@ -613,7 +613,7 @@
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>Медіана часу від початку аномалії до її фіксації: база 288 год (П), ціль: медіана не більше 2 год за 3 міс. пілоту; додатковий контроль хвоста розподілу: P80 не більше 4 год</t>
+          <t>Медіана часу від початку аномалії до її фіксації: база (медіана і середнє) 288 год (П), ціль: медіана не більше 2 год за 3 міс. пілоту; додатковий контроль хвоста розподілу: P80 не більше 4 год</t>
         </is>
       </c>
     </row>
@@ -1004,7 +1004,7 @@
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>частину виявляють обходом, решту після рахунку</t>
+          <t>середнє і медіана прийняті рівними 12 добам</t>
         </is>
       </c>
     </row>
@@ -2481,7 +2481,7 @@
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Аналіз історичних 15-хв даних 3 будівель і розмітка аномалій</t>
+          <t>Аналіз історичних погодинних даних комерційного обліку по вводу 3 будівель і розмітка аномалій</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Lab 1 review fixes: per building support versus fixed support and onboarding, A5 timeline aligned with lab 3, median basis, A1 wording
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/lab1/out/lab1_passport_model.xlsx
+++ b/lab1/out/lab1_passport_model.xlsx
@@ -553,7 +553,7 @@
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Енергоменеджер багатоорендного офісного центру виявляє аномальне споживання із запізненням (обходи, погодинні дані вводу або лише місячний рахунок): середнє і медіана 12 діб (П); причину перевитрат встановити складно, бо субоблік знімають вручну раз на місяць, а погодинні дані є лише по вводу, без інтервальних даних по точках обліку. Втрати від аномалій оцінено в 3,4% річного споживання (П).</t>
+          <t>Енергоменеджер багатоорендного офісного центру виявляє аномальне споживання із запізненням (обходи, погодинні дані вводу або лише місячний рахунок): у середньому 12 діб, медіана близько 11 діб, для бази округлена до 12 діб (П); причину перевитрат встановити складно, бо субоблік знімають вручну раз на місяць, а погодинні дані є лише по вводу, без інтервальних даних по точках обліку. Втрати від аномалій оцінено в 3,4% річного споживання (П).</t>
         </is>
       </c>
     </row>
@@ -613,7 +613,7 @@
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>Медіана часу від початку аномалії до її фіксації: база (медіана і середнє) 288 год (П), ціль: медіана не більше 2 год за 3 міс. пілоту; додатковий контроль хвоста розподілу: P80 не більше 4 год</t>
+          <t>Медіана часу від початку аномалії до її фіксації: база 288 год (12 діб; медіана близько 11 діб, округлено, П), ціль: медіана не більше 2 год за 3 міс. пілоту; додатковий контроль хвоста розподілу: P80 не більше 4 год</t>
         </is>
       </c>
     </row>
@@ -637,7 +637,7 @@
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>A1: аномалії, які усуваються після рахунку, становлять не менше 2% річного споживання будівлі (вплив 5, невизначеність 4)</t>
+          <t>A1: втрати від аномалій, які зараз виявляють із запізненням (обходи, погодинні дані, рахунок), становлять не менше 2% річного споживання будівлі (вплив 5, невизначеність 4)</t>
         </is>
       </c>
     </row>
@@ -1004,7 +1004,7 @@
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>середнє і медіана прийняті рівними 12 добам</t>
+          <t>середнє 12,2 доби, медіана близько 11 діб; обидва округлено до 12 діб</t>
         </is>
       </c>
     </row>
@@ -2518,7 +2518,7 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>Прототип шлюзу: мінікомп'ютер, адаптер RS-485, LTE модем</t>
+          <t>Тест A5: тимчасова збірка шлюзу (мінікомп'ютер, адаптер RS-485) в 1 будівлі на 2 тижні</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
@@ -2851,7 +2851,7 @@
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>Онбординг будівлі і підтримка</t>
+          <t>Підтримка будівлі: консультації клієнта, перевірка нестабільних лічильників (у v)</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
@@ -2888,12 +2888,12 @@
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>Супровід: виправлення, оновлення залежностей, нові моделі лічильників</t>
+          <t>Support і change команди: чергування, онбординг нових будівель, виправлення, оновлення, нові моделі лічильників</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>кількість змін і моделей лічильників</t>
+          <t>частки FTE команди супроводу; кількість змін</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr">
@@ -3552,7 +3552,7 @@
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>Аномалії, які усуваються після рахунку, становлять не менше 2% річного споживання будівлі</t>
+          <t>Втрати від аномалій, які зараз виявляють із запізненням (обходи, погодинні дані, рахунок), становлять не менше 2% річного споживання будівлі</t>
         </is>
       </c>
       <c r="D2" s="3" t="n">

</xml_diff>

<commit_message>
Remove forward references between labs: lab 1 assumption tests stated within lab 1, scale trigger counts free pilot buildings, lab 5 checks the trigger with pilots
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/lab1/out/lab1_passport_model.xlsx
+++ b/lab1/out/lab1_passport_model.xlsx
@@ -1364,7 +1364,7 @@
       </c>
       <c r="F23" s="2" t="inlineStr">
         <is>
-          <t>умова варіанта ЛР № 4 і № 5</t>
+          <t>рядок варіанта 14 методичних вказівок до наступних робіт курсу</t>
         </is>
       </c>
     </row>
@@ -1394,7 +1394,7 @@
       </c>
       <c r="F24" s="2" t="inlineStr">
         <is>
-          <t>умова варіанта ЛР № 4 і № 5</t>
+          <t>рядок варіанта 14 методичних вказівок до наступних робіт курсу</t>
         </is>
       </c>
     </row>
@@ -1424,7 +1424,7 @@
       </c>
       <c r="F25" s="2" t="inlineStr">
         <is>
-          <t>умова варіанта ЛР № 4 і № 5: BA/PM, 2 розробники, QA, DevOps</t>
+          <t>рядок варіанта 14 методичних вказівок до наступних робіт курсу: BA/PM, 2 розробники, QA, DevOps</t>
         </is>
       </c>
     </row>

</xml_diff>